<commit_message>
feat: posicao nova/encerrada passa a percentual (3% do PL), calibrado no dado real
Decisao do dono: percentual, sem valor nominal. O piso antigo de R$ 5 mil disparava 329 eventos por mes no dado real de maio a junho (rotacao rotineira). Com 3% do PL: 52 encerradas + 34 novas, fila comercial de 110 por mes. Fixtures ajustadas para as historias continuarem disparando acima do novo limiar.

Co-Authored-By: Claude <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/audit-engine/tests/fixtures-sinteticos/diarios/posicao-2026-08-12.xlsx
+++ b/audit-engine/tests/fixtures-sinteticos/diarios/posicao-2026-08-12.xlsx
@@ -501,10 +501,10 @@
         <v>5</v>
       </c>
       <c r="C5">
-        <v>460000</v>
+        <v>500000</v>
       </c>
       <c r="D5">
-        <v>460000</v>
+        <v>500000</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
@@ -529,10 +529,10 @@
         <v>4</v>
       </c>
       <c r="C7">
-        <v>10000</v>
+        <v>50000</v>
       </c>
       <c r="D7">
-        <v>10000</v>
+        <v>50000</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.25">
@@ -629,10 +629,10 @@
         <v>15</v>
       </c>
       <c r="C15">
-        <v>1020000</v>
+        <v>1060000</v>
       </c>
       <c r="D15">
-        <v>1020000</v>
+        <v>1060000</v>
       </c>
     </row>
   </sheetData>

</xml_diff>